<commit_message>
fix luong HRC1 slab
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC1_BBGN_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC1_BBGN_PhoiTam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CB7B90FE-9333-452B-B07D-119A6B8B9B42}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B25506A-430D-41D0-BD70-40A1E1433397}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -154,6 +154,12 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -165,12 +171,6 @@
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="right" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -194,184 +194,45 @@
   <xdr:twoCellAnchor editAs="oneCell">
     <xdr:from>
       <xdr:col>0</xdr:col>
-      <xdr:colOff>0</xdr:colOff>
+      <xdr:colOff>89647</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>0</xdr:rowOff>
+      <xdr:rowOff>11206</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>1</xdr:col>
-      <xdr:colOff>1645583</xdr:colOff>
+      <xdr:colOff>1265953</xdr:colOff>
       <xdr:row>1</xdr:row>
-      <xdr:rowOff>605118</xdr:rowOff>
+      <xdr:rowOff>544707</xdr:rowOff>
     </xdr:to>
-    <xdr:grpSp>
-      <xdr:nvGrpSpPr>
-        <xdr:cNvPr id="8" name="Group 3">
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{5F61B5B9-D8A8-4768-88EC-8F1FB8FBA6EB}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{C0571BD1-64CC-43BD-A99C-775741C5186E}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
-        <xdr:cNvGrpSpPr>
-          <a:grpSpLocks noChangeAspect="1"/>
-        </xdr:cNvGrpSpPr>
-      </xdr:nvGrpSpPr>
-      <xdr:grpSpPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
         <a:xfrm>
-          <a:off x="0" y="0"/>
-          <a:ext cx="2250701" cy="795618"/>
-          <a:chOff x="0" y="1"/>
-          <a:chExt cx="2095500" cy="876300"/>
+          <a:off x="89647" y="11206"/>
+          <a:ext cx="1781424" cy="724001"/>
         </a:xfrm>
-      </xdr:grpSpPr>
-      <xdr:pic>
-        <xdr:nvPicPr>
-          <xdr:cNvPr id="9" name="Picture 6">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{CEC04943-C9AA-4BE5-929A-6C08E7A8321A}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvPicPr>
-            <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-          </xdr:cNvPicPr>
-        </xdr:nvPicPr>
-        <xdr:blipFill>
-          <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1" cstate="print">
-            <a:extLst>
-              <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-                <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-              </a:ext>
-            </a:extLst>
-          </a:blip>
-          <a:srcRect/>
-          <a:stretch>
-            <a:fillRect/>
-          </a:stretch>
-        </xdr:blipFill>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="133350" y="1"/>
-            <a:ext cx="1819275" cy="407343"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-          <a:extLst>
-            <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-              <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-                <a:solidFill>
-                  <a:srgbClr val="FFFFFF"/>
-                </a:solidFill>
-              </a14:hiddenFill>
-            </a:ext>
-            <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-              <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:miter lim="800000"/>
-                <a:headEnd/>
-                <a:tailEnd/>
-              </a14:hiddenLine>
-            </a:ext>
-          </a:extLst>
-        </xdr:spPr>
-      </xdr:pic>
-      <xdr:sp macro="" textlink="">
-        <xdr:nvSpPr>
-          <xdr:cNvPr id="10" name="TextBox 4">
-            <a:extLst>
-              <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-                <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{46EABE90-C3B5-4394-8961-5E731E42E45A}"/>
-              </a:ext>
-            </a:extLst>
-          </xdr:cNvPr>
-          <xdr:cNvSpPr txBox="1">
-            <a:spLocks noChangeArrowheads="1"/>
-          </xdr:cNvSpPr>
-        </xdr:nvSpPr>
-        <xdr:spPr>
-          <a:xfrm>
-            <a:off x="0" y="382217"/>
-            <a:ext cx="2095500" cy="494084"/>
-          </a:xfrm>
-          <a:prstGeom prst="rect">
-            <a:avLst/>
-          </a:prstGeom>
-          <a:noFill/>
-          <a:ln>
-            <a:noFill/>
-          </a:ln>
-        </xdr:spPr>
-        <xdr:txBody>
-          <a:bodyPr rot="0" vert="horz" wrap="square" lIns="91440" tIns="45720" rIns="91440" bIns="45720" anchor="ctr" anchorCtr="0" upright="1">
-            <a:noAutofit/>
-          </a:bodyPr>
-          <a:lstStyle/>
-          <a:p>
-            <a:pPr marL="0" marR="0" algn="ctr">
-              <a:lnSpc>
-                <a:spcPts val="1200"/>
-              </a:lnSpc>
-              <a:spcBef>
-                <a:spcPts val="0"/>
-              </a:spcBef>
-              <a:spcAft>
-                <a:spcPts val="800"/>
-              </a:spcAft>
-            </a:pPr>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst/>
-                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              </a:rPr>
-              <a:t>CÔNG TY CỔ PHẦN THÉP</a:t>
-            </a:r>
-            <a:br>
-              <a:rPr lang="en-US" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst/>
-                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              </a:rPr>
-            </a:br>
-            <a:r>
-              <a:rPr lang="en-US" sz="1200" b="1">
-                <a:solidFill>
-                  <a:srgbClr val="000000"/>
-                </a:solidFill>
-                <a:effectLst/>
-                <a:latin typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-                <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-                <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-              </a:rPr>
-              <a:t>HÒA PHÁT DUNG QUẤT</a:t>
-            </a:r>
-            <a:endParaRPr lang="en-US" sz="1100">
-              <a:effectLst/>
-              <a:latin typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:ea typeface="Calibri" panose="020F0502020204030204" pitchFamily="34" charset="0"/>
-              <a:cs typeface="Times New Roman" panose="02020603050405020304" pitchFamily="18" charset="0"/>
-            </a:endParaRPr>
-          </a:p>
-        </xdr:txBody>
-      </xdr:sp>
-    </xdr:grpSp>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
     <xdr:clientData/>
   </xdr:twoCellAnchor>
 </xdr:wsDr>
@@ -678,7 +539,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="27" style="10" customWidth="1"/>
+    <col min="2" max="2" width="27" style="6" customWidth="1"/>
     <col min="3" max="3" width="49.42578125" style="2" customWidth="1"/>
     <col min="4" max="4" width="21.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
@@ -692,39 +553,39 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="9" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="8"/>
-      <c r="C1" s="8"/>
-      <c r="D1" s="8"/>
-      <c r="E1" s="8"/>
-      <c r="F1" s="8"/>
-      <c r="G1" s="8"/>
+      <c r="B1" s="10"/>
+      <c r="C1" s="10"/>
+      <c r="D1" s="10"/>
+      <c r="E1" s="10"/>
+      <c r="F1" s="10"/>
+      <c r="G1" s="10"/>
     </row>
     <row r="2" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="8"/>
-      <c r="B2" s="8"/>
-      <c r="C2" s="8"/>
-      <c r="D2" s="8"/>
-      <c r="E2" s="8"/>
-      <c r="F2" s="8"/>
-      <c r="G2" s="8"/>
+      <c r="A2" s="10"/>
+      <c r="B2" s="10"/>
+      <c r="C2" s="10"/>
+      <c r="D2" s="10"/>
+      <c r="E2" s="10"/>
+      <c r="F2" s="10"/>
+      <c r="G2" s="10"/>
     </row>
     <row r="3" spans="1:7" ht="35.25" x14ac:dyDescent="0.5">
-      <c r="A3" s="5" t="s">
+      <c r="A3" s="7" t="s">
         <v>7</v>
       </c>
-      <c r="B3" s="6"/>
-      <c r="C3" s="6"/>
-      <c r="D3" s="6"/>
-      <c r="E3" s="6"/>
-      <c r="F3" s="6"/>
-      <c r="G3" s="6"/>
+      <c r="B3" s="8"/>
+      <c r="C3" s="8"/>
+      <c r="D3" s="8"/>
+      <c r="E3" s="8"/>
+      <c r="F3" s="8"/>
+      <c r="G3" s="8"/>
     </row>
     <row r="4" spans="1:7" ht="35.25" x14ac:dyDescent="0.5">
       <c r="A4" s="3"/>
-      <c r="B4" s="9"/>
+      <c r="B4" s="5"/>
       <c r="C4" s="4"/>
       <c r="D4" s="4"/>
       <c r="E4" s="4"/>

</xml_diff>

<commit_message>
thêm thông tin người xác nhận
</commit_message>
<xml_diff>
--- a/dataproduct.api/wwwroot/templates/HRC1_BBGN_PhoiTam.xlsx
+++ b/dataproduct.api/wwwroot/templates/HRC1_BBGN_PhoiTam.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\_Projects\BIEUMAU_SANXUAT\Source\dataproduct.BE\dataproduct.api\wwwroot\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0229EA1C-2565-4A2E-9B25-CD57F538C129}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{81728D6F-433D-49BA-912E-2FD3AC96BE78}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="24720" windowHeight="11805" xr2:uid="{8D26054B-D371-44B9-99F0-3A3B1380D846}"/>
   </bookViews>
@@ -60,7 +60,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="6" x14ac:knownFonts="1">
+  <fonts count="8" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -95,6 +95,21 @@
     </font>
     <font>
       <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <b/>
+      <i/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Times New Roman"/>
+      <family val="1"/>
+    </font>
+    <font>
+      <i/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Times New Roman"/>
@@ -115,7 +130,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -138,39 +153,45 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="right" vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -201,8 +222,8 @@
     <xdr:to>
       <xdr:col>1</xdr:col>
       <xdr:colOff>1265953</xdr:colOff>
-      <xdr:row>1</xdr:row>
-      <xdr:rowOff>544707</xdr:rowOff>
+      <xdr:row>0</xdr:row>
+      <xdr:rowOff>735207</xdr:rowOff>
     </xdr:to>
     <xdr:pic>
       <xdr:nvPicPr>
@@ -539,7 +560,7 @@
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="9.140625" style="2"/>
-    <col min="2" max="2" width="27" style="6" customWidth="1"/>
+    <col min="2" max="2" width="27" style="3" customWidth="1"/>
     <col min="3" max="3" width="49.42578125" style="2" customWidth="1"/>
     <col min="4" max="4" width="21.85546875" style="2" customWidth="1"/>
     <col min="5" max="5" width="20.7109375" style="2" customWidth="1"/>
@@ -552,45 +573,45 @@
     <col min="13" max="16384" width="9.140625" style="2"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+    <row r="1" spans="1:7" ht="65.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="6" t="s">
         <v>8</v>
       </c>
-      <c r="B1" s="10"/>
-      <c r="C1" s="10"/>
-      <c r="D1" s="10"/>
-      <c r="E1" s="10"/>
-      <c r="F1" s="10"/>
-      <c r="G1" s="10"/>
+      <c r="B1" s="6"/>
+      <c r="C1" s="6"/>
+      <c r="D1" s="6"/>
+      <c r="E1" s="6"/>
+      <c r="F1" s="6"/>
+      <c r="G1" s="6"/>
     </row>
-    <row r="2" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="10"/>
-      <c r="B2" s="10"/>
-      <c r="C2" s="10"/>
-      <c r="D2" s="10"/>
-      <c r="E2" s="10"/>
-      <c r="F2" s="10"/>
-      <c r="G2" s="10"/>
+    <row r="2" spans="1:7" ht="64.5" customHeight="1" x14ac:dyDescent="0.5">
+      <c r="A2" s="7" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" s="8"/>
+      <c r="C2" s="8"/>
+      <c r="D2" s="8"/>
+      <c r="E2" s="8"/>
+      <c r="F2" s="8"/>
+      <c r="G2" s="8"/>
     </row>
-    <row r="3" spans="1:7" ht="35.25" x14ac:dyDescent="0.5">
-      <c r="A3" s="7" t="s">
-        <v>7</v>
-      </c>
-      <c r="B3" s="8"/>
-      <c r="C3" s="8"/>
-      <c r="D3" s="8"/>
-      <c r="E3" s="8"/>
-      <c r="F3" s="8"/>
-      <c r="G3" s="8"/>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" s="4"/>
+      <c r="B3" s="5"/>
+      <c r="C3" s="5"/>
+      <c r="D3" s="5"/>
+      <c r="E3" s="5"/>
+      <c r="F3" s="5"/>
+      <c r="G3" s="5"/>
     </row>
-    <row r="4" spans="1:7" ht="35.25" x14ac:dyDescent="0.5">
-      <c r="A4" s="3"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="4"/>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
-      <c r="F4" s="4"/>
-      <c r="G4" s="4"/>
+    <row r="4" spans="1:7" ht="35.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="9"/>
+      <c r="B4" s="9"/>
+      <c r="C4" s="9"/>
+      <c r="D4" s="9"/>
+      <c r="E4" s="9"/>
+      <c r="F4" s="9"/>
+      <c r="G4" s="9"/>
     </row>
     <row r="5" spans="1:7" ht="15.75" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
@@ -616,9 +637,11 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="4">
     <mergeCell ref="A3:G3"/>
-    <mergeCell ref="A1:G2"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A2:G2"/>
+    <mergeCell ref="A4:G4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" verticalDpi="0" r:id="rId1"/>

</xml_diff>